<commit_message>
remove personal metadata from template xlsx
</commit_message>
<xml_diff>
--- a/resources/templates/Submission template v20.xlsx
+++ b/resources/templates/Submission template v20.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/suyya/Workspace/senior-accounting-officer-submission-frontend/resources/templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A21D53D-0654-0146-9ECB-977C5D1B1529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAEEC74-33FC-4142-8ACB-A59373C55709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="660" windowWidth="30240" windowHeight="17640" xr2:uid="{385E0F26-D714-DE43-8BBA-8E250D50B1AF}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17640" xr2:uid="{385E0F26-D714-DE43-8BBA-8E250D50B1AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Submission template" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
SAOD-1156 fix template dropdown issue
</commit_message>
<xml_diff>
--- a/resources/templates/Submission template v20.xlsx
+++ b/resources/templates/Submission template v20.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAEEC74-33FC-4142-8ACB-A59373C55709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD4C462-5C8C-634C-AD49-866DDBA7CF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17640" xr2:uid="{385E0F26-D714-DE43-8BBA-8E250D50B1AF}"/>
   </bookViews>
@@ -1990,7 +1990,7 @@
       <formula1>"LTD,PLC"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E14" xr:uid="{E23A466F-0C81-4900-87B5-29016B8D0684}">
-      <formula1>"Active,Administration ,Dormant,Liquidation"</formula1>
+      <formula1>"Active,Administration,Dormant,Liquidation"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q14" xr:uid="{0143D42B-EC96-4CF7-AEE3-EB19D97195E0}"/>
   </dataValidations>

</xml_diff>

<commit_message>
SAOD-1156 fix template dropdown issue (#206)
Co-authored-by: Su-Yang Yu <20665693+suyangyu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resources/templates/Submission template v20.xlsx
+++ b/resources/templates/Submission template v20.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAEEC74-33FC-4142-8ACB-A59373C55709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD4C462-5C8C-634C-AD49-866DDBA7CF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17640" xr2:uid="{385E0F26-D714-DE43-8BBA-8E250D50B1AF}"/>
   </bookViews>
@@ -1990,7 +1990,7 @@
       <formula1>"LTD,PLC"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E14" xr:uid="{E23A466F-0C81-4900-87B5-29016B8D0684}">
-      <formula1>"Active,Administration ,Dormant,Liquidation"</formula1>
+      <formula1>"Active,Administration,Dormant,Liquidation"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q14" xr:uid="{0143D42B-EC96-4CF7-AEE3-EB19D97195E0}"/>
   </dataValidations>

</xml_diff>